<commit_message>
feat: Add Tay chatbot (Claude API), proposal restructure & supporting docs
- Tay chatbot: Express proxy server with Claude Sonnet API, section-aware
  context, conversation history, concise response tuning
- Interactive Pitch: new Section 02 (Operating Paradigm), updated suggestions
  per section, larger chat panel, removed date references from CTAs
- New files: Team Roles, Tech Lead Profile, Full Pitch EDITABLE DOCX,
  INTAKE/Full Pitch DOCX generators, Transformation Roadmap XLSX
- Updated bibliography, Strategic Pitch (HTML/DOCX/PPTX), .gitignore (.env)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Taylor Group/proposal-2.0/pitch/Taylor-Group-Transformation-Roadmap.xlsx
+++ b/Taylor Group/proposal-2.0/pitch/Taylor-Group-Transformation-Roadmap.xlsx
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -203,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -233,11 +232,55 @@
         <color rgb="001A1A2E"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D5D5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D5D5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D5D5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D5D5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D5D5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D5D5"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D5D5"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D5D5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -273,7 +316,7 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -309,7 +352,7 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -348,7 +391,7 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -390,7 +433,7 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -426,7 +469,7 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -516,6 +559,23 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -991,21 +1051,21 @@
           <t>PHASE 0 — PRE-ENGAGEMENT</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
+      <c r="B2" s="107" t="n"/>
+      <c r="C2" s="107" t="n"/>
+      <c r="D2" s="107" t="n"/>
+      <c r="E2" s="107" t="n"/>
+      <c r="F2" s="107" t="n"/>
+      <c r="G2" s="107" t="n"/>
+      <c r="H2" s="107" t="n"/>
+      <c r="I2" s="107" t="n"/>
+      <c r="J2" s="107" t="n"/>
+      <c r="K2" s="107" t="n"/>
+      <c r="L2" s="107" t="n"/>
+      <c r="M2" s="107" t="n"/>
+      <c r="N2" s="107" t="n"/>
+      <c r="O2" s="107" t="n"/>
+      <c r="P2" s="108" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="4" t="n">
@@ -1066,10 +1126,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M3" s="13" t="n">
+      <c r="M3" s="109" t="n">
         <v>46099</v>
       </c>
-      <c r="N3" s="13" t="n">
+      <c r="N3" s="109" t="n">
         <v>46103</v>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -1141,10 +1201,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M4" s="13" t="n">
+      <c r="M4" s="109" t="n">
         <v>46101</v>
       </c>
-      <c r="N4" s="13" t="n">
+      <c r="N4" s="109" t="n">
         <v>46106</v>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -1216,10 +1276,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M5" s="13" t="n">
+      <c r="M5" s="109" t="n">
         <v>46103</v>
       </c>
-      <c r="N5" s="13" t="n">
+      <c r="N5" s="109" t="n">
         <v>46108</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
@@ -1291,10 +1351,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M6" s="13" t="n">
+      <c r="M6" s="109" t="n">
         <v>46106</v>
       </c>
-      <c r="N6" s="13" t="n">
+      <c r="N6" s="109" t="n">
         <v>46112</v>
       </c>
       <c r="O6" s="4" t="inlineStr">
@@ -1366,10 +1426,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M7" s="13" t="n">
+      <c r="M7" s="109" t="n">
         <v>46109</v>
       </c>
-      <c r="N7" s="13" t="n">
+      <c r="N7" s="109" t="n">
         <v>46114</v>
       </c>
       <c r="O7" s="4" t="inlineStr">
@@ -1441,10 +1501,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M8" s="13" t="n">
+      <c r="M8" s="109" t="n">
         <v>46114</v>
       </c>
-      <c r="N8" s="13" t="n">
+      <c r="N8" s="109" t="n">
         <v>46117</v>
       </c>
       <c r="O8" s="4" t="inlineStr">
@@ -1516,10 +1576,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M9" s="13" t="n">
+      <c r="M9" s="109" t="n">
         <v>46106</v>
       </c>
-      <c r="N9" s="13" t="n">
+      <c r="N9" s="109" t="n">
         <v>46111</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
@@ -1591,10 +1651,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M10" s="13" t="n">
+      <c r="M10" s="109" t="n">
         <v>46108</v>
       </c>
-      <c r="N10" s="13" t="n">
+      <c r="N10" s="109" t="n">
         <v>46114</v>
       </c>
       <c r="O10" s="4" t="inlineStr">
@@ -1666,10 +1726,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M11" s="13" t="n">
+      <c r="M11" s="109" t="n">
         <v>46111</v>
       </c>
-      <c r="N11" s="13" t="n">
+      <c r="N11" s="109" t="n">
         <v>46115</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
@@ -1741,10 +1801,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M12" s="13" t="n">
+      <c r="M12" s="109" t="n">
         <v>46111</v>
       </c>
-      <c r="N12" s="13" t="n">
+      <c r="N12" s="109" t="n">
         <v>46116</v>
       </c>
       <c r="O12" s="4" t="inlineStr">
@@ -1816,10 +1876,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M13" s="13" t="n">
+      <c r="M13" s="109" t="n">
         <v>46113</v>
       </c>
-      <c r="N13" s="13" t="n">
+      <c r="N13" s="109" t="n">
         <v>46117</v>
       </c>
       <c r="O13" s="4" t="inlineStr">
@@ -1891,10 +1951,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M14" s="13" t="n">
+      <c r="M14" s="109" t="n">
         <v>46113</v>
       </c>
-      <c r="N14" s="13" t="n">
+      <c r="N14" s="109" t="n">
         <v>46118</v>
       </c>
       <c r="O14" s="4" t="inlineStr">
@@ -1966,10 +2026,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M15" s="13" t="n">
+      <c r="M15" s="109" t="n">
         <v>46114</v>
       </c>
-      <c r="N15" s="13" t="n">
+      <c r="N15" s="109" t="n">
         <v>46119</v>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -2041,10 +2101,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M16" s="13" t="n">
+      <c r="M16" s="109" t="n">
         <v>46109</v>
       </c>
-      <c r="N16" s="13" t="n">
+      <c r="N16" s="109" t="n">
         <v>46114</v>
       </c>
       <c r="O16" s="4" t="inlineStr">
@@ -2116,10 +2176,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M17" s="13" t="n">
+      <c r="M17" s="109" t="n">
         <v>46113</v>
       </c>
-      <c r="N17" s="13" t="n">
+      <c r="N17" s="109" t="n">
         <v>46118</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
@@ -2191,10 +2251,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M18" s="13" t="n">
+      <c r="M18" s="109" t="n">
         <v>46115</v>
       </c>
-      <c r="N18" s="13" t="n">
+      <c r="N18" s="109" t="n">
         <v>46120</v>
       </c>
       <c r="O18" s="4" t="inlineStr">
@@ -2266,10 +2326,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M19" s="13" t="n">
+      <c r="M19" s="109" t="n">
         <v>46106</v>
       </c>
-      <c r="N19" s="13" t="n">
+      <c r="N19" s="109" t="n">
         <v>46111</v>
       </c>
       <c r="O19" s="4" t="inlineStr">
@@ -2341,10 +2401,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M20" s="13" t="n">
+      <c r="M20" s="109" t="n">
         <v>46111</v>
       </c>
-      <c r="N20" s="13" t="n">
+      <c r="N20" s="109" t="n">
         <v>46117</v>
       </c>
       <c r="O20" s="4" t="inlineStr">
@@ -2416,10 +2476,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M21" s="13" t="n">
+      <c r="M21" s="109" t="n">
         <v>46117</v>
       </c>
-      <c r="N21" s="13" t="n">
+      <c r="N21" s="109" t="n">
         <v>46124</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
@@ -2491,10 +2551,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M22" s="13" t="n">
+      <c r="M22" s="109" t="n">
         <v>46122</v>
       </c>
-      <c r="N22" s="13" t="n">
+      <c r="N22" s="109" t="n">
         <v>46127</v>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -2513,21 +2573,21 @@
           <t>PHASE 1 — INTAKE (Remote)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
-      <c r="P23" s="3" t="n"/>
+      <c r="B23" s="107" t="n"/>
+      <c r="C23" s="107" t="n"/>
+      <c r="D23" s="107" t="n"/>
+      <c r="E23" s="107" t="n"/>
+      <c r="F23" s="107" t="n"/>
+      <c r="G23" s="107" t="n"/>
+      <c r="H23" s="107" t="n"/>
+      <c r="I23" s="107" t="n"/>
+      <c r="J23" s="107" t="n"/>
+      <c r="K23" s="107" t="n"/>
+      <c r="L23" s="107" t="n"/>
+      <c r="M23" s="107" t="n"/>
+      <c r="N23" s="107" t="n"/>
+      <c r="O23" s="107" t="n"/>
+      <c r="P23" s="108" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="17" t="n">
@@ -2588,11 +2648,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M24" s="25" t="n">
+      <c r="M24" s="110" t="n">
         <v>46143</v>
       </c>
-      <c r="N24" s="25" t="n">
-        <v>46145</v>
+      <c r="N24" s="110" t="n">
+        <v>46147</v>
       </c>
       <c r="O24" s="17" t="inlineStr">
         <is>
@@ -2663,11 +2723,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M25" s="25" t="n">
-        <v>46144</v>
-      </c>
-      <c r="N25" s="25" t="n">
-        <v>46147</v>
+      <c r="M25" s="110" t="n">
+        <v>46145</v>
+      </c>
+      <c r="N25" s="110" t="n">
+        <v>46151</v>
       </c>
       <c r="O25" s="17" t="inlineStr">
         <is>
@@ -2738,11 +2798,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M26" s="25" t="n">
+      <c r="M26" s="110" t="n">
         <v>46143</v>
       </c>
-      <c r="N26" s="25" t="n">
-        <v>46146</v>
+      <c r="N26" s="110" t="n">
+        <v>46149</v>
       </c>
       <c r="O26" s="17" t="inlineStr">
         <is>
@@ -2813,11 +2873,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M27" s="25" t="n">
-        <v>46146</v>
-      </c>
-      <c r="N27" s="25" t="n">
-        <v>46147</v>
+      <c r="M27" s="110" t="n">
+        <v>46149</v>
+      </c>
+      <c r="N27" s="110" t="n">
+        <v>46151</v>
       </c>
       <c r="O27" s="17" t="inlineStr">
         <is>
@@ -2888,11 +2948,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M28" s="25" t="n">
-        <v>46147</v>
-      </c>
-      <c r="N28" s="25" t="n">
-        <v>46157</v>
+      <c r="M28" s="110" t="n">
+        <v>46151</v>
+      </c>
+      <c r="N28" s="110" t="n">
+        <v>46172</v>
       </c>
       <c r="O28" s="17" t="inlineStr">
         <is>
@@ -2963,11 +3023,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M29" s="25" t="n">
-        <v>46147</v>
-      </c>
-      <c r="N29" s="25" t="n">
-        <v>46154</v>
+      <c r="M29" s="110" t="n">
+        <v>46151</v>
+      </c>
+      <c r="N29" s="110" t="n">
+        <v>46166</v>
       </c>
       <c r="O29" s="17" t="inlineStr">
         <is>
@@ -3038,11 +3098,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M30" s="25" t="n">
-        <v>46147</v>
-      </c>
-      <c r="N30" s="25" t="n">
-        <v>46154</v>
+      <c r="M30" s="110" t="n">
+        <v>46151</v>
+      </c>
+      <c r="N30" s="110" t="n">
+        <v>46166</v>
       </c>
       <c r="O30" s="17" t="inlineStr">
         <is>
@@ -3113,11 +3173,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M31" s="25" t="n">
-        <v>46147</v>
-      </c>
-      <c r="N31" s="25" t="n">
-        <v>46157</v>
+      <c r="M31" s="110" t="n">
+        <v>46151</v>
+      </c>
+      <c r="N31" s="110" t="n">
+        <v>46172</v>
       </c>
       <c r="O31" s="17" t="inlineStr">
         <is>
@@ -3188,11 +3248,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M32" s="25" t="n">
-        <v>46149</v>
-      </c>
-      <c r="N32" s="25" t="n">
-        <v>46157</v>
+      <c r="M32" s="110" t="n">
+        <v>46155</v>
+      </c>
+      <c r="N32" s="110" t="n">
+        <v>46172</v>
       </c>
       <c r="O32" s="17" t="inlineStr">
         <is>
@@ -3263,11 +3323,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M33" s="25" t="n">
-        <v>46147</v>
-      </c>
-      <c r="N33" s="25" t="n">
-        <v>46152</v>
+      <c r="M33" s="110" t="n">
+        <v>46151</v>
+      </c>
+      <c r="N33" s="110" t="n">
+        <v>46162</v>
       </c>
       <c r="O33" s="17" t="inlineStr">
         <is>
@@ -3338,11 +3398,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M34" s="25" t="n">
-        <v>46148</v>
-      </c>
-      <c r="N34" s="25" t="n">
-        <v>46157</v>
+      <c r="M34" s="110" t="n">
+        <v>46153</v>
+      </c>
+      <c r="N34" s="110" t="n">
+        <v>46172</v>
       </c>
       <c r="O34" s="17" t="inlineStr">
         <is>
@@ -3413,11 +3473,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M35" s="25" t="n">
-        <v>46150</v>
-      </c>
-      <c r="N35" s="25" t="n">
+      <c r="M35" s="110" t="n">
         <v>46157</v>
+      </c>
+      <c r="N35" s="110" t="n">
+        <v>46172</v>
       </c>
       <c r="O35" s="17" t="inlineStr">
         <is>
@@ -3488,11 +3548,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M36" s="25" t="n">
-        <v>46150</v>
-      </c>
-      <c r="N36" s="25" t="n">
+      <c r="M36" s="110" t="n">
         <v>46157</v>
+      </c>
+      <c r="N36" s="110" t="n">
+        <v>46172</v>
       </c>
       <c r="O36" s="17" t="inlineStr">
         <is>
@@ -3563,11 +3623,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M37" s="25" t="n">
-        <v>46150</v>
-      </c>
-      <c r="N37" s="25" t="n">
-        <v>46162</v>
+      <c r="M37" s="110" t="n">
+        <v>46157</v>
+      </c>
+      <c r="N37" s="110" t="n">
+        <v>46182</v>
       </c>
       <c r="O37" s="17" t="inlineStr">
         <is>
@@ -3638,11 +3698,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M38" s="25" t="n">
-        <v>46150</v>
-      </c>
-      <c r="N38" s="25" t="n">
-        <v>46160</v>
+      <c r="M38" s="110" t="n">
+        <v>46157</v>
+      </c>
+      <c r="N38" s="110" t="n">
+        <v>46178</v>
       </c>
       <c r="O38" s="17" t="inlineStr">
         <is>
@@ -3713,11 +3773,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M39" s="25" t="n">
-        <v>46152</v>
-      </c>
-      <c r="N39" s="25" t="n">
+      <c r="M39" s="110" t="n">
         <v>46162</v>
+      </c>
+      <c r="N39" s="110" t="n">
+        <v>46182</v>
       </c>
       <c r="O39" s="17" t="inlineStr">
         <is>
@@ -3788,11 +3848,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M40" s="25" t="n">
-        <v>46152</v>
-      </c>
-      <c r="N40" s="25" t="n">
-        <v>46160</v>
+      <c r="M40" s="110" t="n">
+        <v>46162</v>
+      </c>
+      <c r="N40" s="110" t="n">
+        <v>46178</v>
       </c>
       <c r="O40" s="17" t="inlineStr">
         <is>
@@ -3863,11 +3923,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M41" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N41" s="25" t="n">
-        <v>46164</v>
+      <c r="M41" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N41" s="110" t="n">
+        <v>46186</v>
       </c>
       <c r="O41" s="17" t="inlineStr">
         <is>
@@ -3938,11 +3998,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M42" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N42" s="25" t="n">
-        <v>46164</v>
+      <c r="M42" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N42" s="110" t="n">
+        <v>46186</v>
       </c>
       <c r="O42" s="17" t="inlineStr">
         <is>
@@ -4013,11 +4073,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M43" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N43" s="25" t="n">
-        <v>46164</v>
+      <c r="M43" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N43" s="110" t="n">
+        <v>46186</v>
       </c>
       <c r="O43" s="17" t="inlineStr">
         <is>
@@ -4088,11 +4148,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M44" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N44" s="25" t="n">
-        <v>46164</v>
+      <c r="M44" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N44" s="110" t="n">
+        <v>46186</v>
       </c>
       <c r="O44" s="17" t="inlineStr">
         <is>
@@ -4163,11 +4223,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M45" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N45" s="25" t="n">
-        <v>46164</v>
+      <c r="M45" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N45" s="110" t="n">
+        <v>46186</v>
       </c>
       <c r="O45" s="17" t="inlineStr">
         <is>
@@ -4238,11 +4298,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M46" s="25" t="n">
-        <v>46164</v>
-      </c>
-      <c r="N46" s="25" t="n">
-        <v>46170</v>
+      <c r="M46" s="110" t="n">
+        <v>46186</v>
+      </c>
+      <c r="N46" s="110" t="n">
+        <v>46199</v>
       </c>
       <c r="O46" s="17" t="inlineStr">
         <is>
@@ -4313,11 +4373,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M47" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N47" s="25" t="n">
-        <v>46167</v>
+      <c r="M47" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N47" s="110" t="n">
+        <v>46193</v>
       </c>
       <c r="O47" s="17" t="inlineStr">
         <is>
@@ -4388,11 +4448,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M48" s="25" t="n">
-        <v>46157</v>
-      </c>
-      <c r="N48" s="25" t="n">
-        <v>46167</v>
+      <c r="M48" s="110" t="n">
+        <v>46172</v>
+      </c>
+      <c r="N48" s="110" t="n">
+        <v>46193</v>
       </c>
       <c r="O48" s="17" t="inlineStr">
         <is>
@@ -4463,11 +4523,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M49" s="25" t="n">
-        <v>46162</v>
-      </c>
-      <c r="N49" s="25" t="n">
-        <v>46170</v>
+      <c r="M49" s="110" t="n">
+        <v>46182</v>
+      </c>
+      <c r="N49" s="110" t="n">
+        <v>46199</v>
       </c>
       <c r="O49" s="17" t="inlineStr">
         <is>
@@ -4538,11 +4598,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M50" s="25" t="n">
-        <v>46164</v>
-      </c>
-      <c r="N50" s="25" t="n">
-        <v>46170</v>
+      <c r="M50" s="110" t="n">
+        <v>46186</v>
+      </c>
+      <c r="N50" s="110" t="n">
+        <v>46199</v>
       </c>
       <c r="O50" s="17" t="inlineStr">
         <is>
@@ -4613,11 +4673,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M51" s="25" t="n">
-        <v>46167</v>
-      </c>
-      <c r="N51" s="25" t="n">
-        <v>46172</v>
+      <c r="M51" s="110" t="n">
+        <v>46193</v>
+      </c>
+      <c r="N51" s="110" t="n">
+        <v>46203</v>
       </c>
       <c r="O51" s="17" t="inlineStr">
         <is>
@@ -4635,21 +4695,21 @@
           <t>PHASE 2 — DISCOVERY (Onsite Toronto + Remote)</t>
         </is>
       </c>
-      <c r="B52" s="3" t="n"/>
-      <c r="C52" s="3" t="n"/>
-      <c r="D52" s="3" t="n"/>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="n"/>
-      <c r="I52" s="3" t="n"/>
-      <c r="J52" s="3" t="n"/>
-      <c r="K52" s="3" t="n"/>
-      <c r="L52" s="3" t="n"/>
-      <c r="M52" s="3" t="n"/>
-      <c r="N52" s="3" t="n"/>
-      <c r="O52" s="3" t="n"/>
-      <c r="P52" s="3" t="n"/>
+      <c r="B52" s="107" t="n"/>
+      <c r="C52" s="107" t="n"/>
+      <c r="D52" s="107" t="n"/>
+      <c r="E52" s="107" t="n"/>
+      <c r="F52" s="107" t="n"/>
+      <c r="G52" s="107" t="n"/>
+      <c r="H52" s="107" t="n"/>
+      <c r="I52" s="107" t="n"/>
+      <c r="J52" s="107" t="n"/>
+      <c r="K52" s="107" t="n"/>
+      <c r="L52" s="107" t="n"/>
+      <c r="M52" s="107" t="n"/>
+      <c r="N52" s="107" t="n"/>
+      <c r="O52" s="107" t="n"/>
+      <c r="P52" s="108" t="n"/>
     </row>
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="30" t="n">
@@ -4710,11 +4770,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M53" s="38" t="n">
-        <v>46174</v>
-      </c>
-      <c r="N53" s="38" t="n">
-        <v>46178</v>
+      <c r="M53" s="111" t="n">
+        <v>46204</v>
+      </c>
+      <c r="N53" s="111" t="n">
+        <v>46208</v>
       </c>
       <c r="O53" s="30" t="inlineStr">
         <is>
@@ -4785,11 +4845,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M54" s="38" t="n">
-        <v>46175</v>
-      </c>
-      <c r="N54" s="38" t="n">
-        <v>46179</v>
+      <c r="M54" s="111" t="n">
+        <v>46205</v>
+      </c>
+      <c r="N54" s="111" t="n">
+        <v>46209</v>
       </c>
       <c r="O54" s="30" t="inlineStr">
         <is>
@@ -4860,11 +4920,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M55" s="38" t="n">
-        <v>46176</v>
-      </c>
-      <c r="N55" s="38" t="n">
-        <v>46179</v>
+      <c r="M55" s="111" t="n">
+        <v>46206</v>
+      </c>
+      <c r="N55" s="111" t="n">
+        <v>46209</v>
       </c>
       <c r="O55" s="30" t="inlineStr">
         <is>
@@ -4935,11 +4995,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M56" s="38" t="n">
-        <v>46180</v>
-      </c>
-      <c r="N56" s="38" t="n">
-        <v>46180</v>
+      <c r="M56" s="111" t="n">
+        <v>46210</v>
+      </c>
+      <c r="N56" s="111" t="n">
+        <v>46210</v>
       </c>
       <c r="O56" s="30" t="inlineStr">
         <is>
@@ -5010,11 +5070,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M57" s="38" t="n">
-        <v>46180</v>
-      </c>
-      <c r="N57" s="38" t="n">
-        <v>46187</v>
+      <c r="M57" s="111" t="n">
+        <v>46210</v>
+      </c>
+      <c r="N57" s="111" t="n">
+        <v>46217</v>
       </c>
       <c r="O57" s="30" t="inlineStr">
         <is>
@@ -5085,11 +5145,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M58" s="38" t="n">
-        <v>46181</v>
-      </c>
-      <c r="N58" s="38" t="n">
-        <v>46191</v>
+      <c r="M58" s="111" t="n">
+        <v>46211</v>
+      </c>
+      <c r="N58" s="111" t="n">
+        <v>46221</v>
       </c>
       <c r="O58" s="30" t="inlineStr">
         <is>
@@ -5160,11 +5220,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M59" s="38" t="n">
-        <v>46183</v>
-      </c>
-      <c r="N59" s="38" t="n">
-        <v>46191</v>
+      <c r="M59" s="111" t="n">
+        <v>46213</v>
+      </c>
+      <c r="N59" s="111" t="n">
+        <v>46221</v>
       </c>
       <c r="O59" s="30" t="inlineStr">
         <is>
@@ -5235,11 +5295,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M60" s="38" t="n">
-        <v>46181</v>
-      </c>
-      <c r="N60" s="38" t="n">
-        <v>46191</v>
+      <c r="M60" s="111" t="n">
+        <v>46211</v>
+      </c>
+      <c r="N60" s="111" t="n">
+        <v>46221</v>
       </c>
       <c r="O60" s="30" t="inlineStr">
         <is>
@@ -5310,11 +5370,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M61" s="38" t="n">
-        <v>46182</v>
-      </c>
-      <c r="N61" s="38" t="n">
-        <v>46188</v>
+      <c r="M61" s="111" t="n">
+        <v>46212</v>
+      </c>
+      <c r="N61" s="111" t="n">
+        <v>46218</v>
       </c>
       <c r="O61" s="30" t="inlineStr">
         <is>
@@ -5385,11 +5445,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M62" s="38" t="n">
-        <v>46183</v>
-      </c>
-      <c r="N62" s="38" t="n">
-        <v>46189</v>
+      <c r="M62" s="111" t="n">
+        <v>46213</v>
+      </c>
+      <c r="N62" s="111" t="n">
+        <v>46219</v>
       </c>
       <c r="O62" s="30" t="inlineStr">
         <is>
@@ -5460,11 +5520,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M63" s="38" t="n">
-        <v>46182</v>
-      </c>
-      <c r="N63" s="38" t="n">
-        <v>46189</v>
+      <c r="M63" s="111" t="n">
+        <v>46212</v>
+      </c>
+      <c r="N63" s="111" t="n">
+        <v>46219</v>
       </c>
       <c r="O63" s="30" t="inlineStr">
         <is>
@@ -5535,11 +5595,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M64" s="38" t="n">
-        <v>46183</v>
-      </c>
-      <c r="N64" s="38" t="n">
-        <v>46189</v>
+      <c r="M64" s="111" t="n">
+        <v>46213</v>
+      </c>
+      <c r="N64" s="111" t="n">
+        <v>46219</v>
       </c>
       <c r="O64" s="30" t="inlineStr">
         <is>
@@ -5610,11 +5670,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M65" s="38" t="n">
-        <v>46183</v>
-      </c>
-      <c r="N65" s="38" t="n">
-        <v>46191</v>
+      <c r="M65" s="111" t="n">
+        <v>46213</v>
+      </c>
+      <c r="N65" s="111" t="n">
+        <v>46221</v>
       </c>
       <c r="O65" s="30" t="inlineStr">
         <is>
@@ -5685,11 +5745,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M66" s="38" t="n">
-        <v>46185</v>
-      </c>
-      <c r="N66" s="38" t="n">
-        <v>46191</v>
+      <c r="M66" s="111" t="n">
+        <v>46215</v>
+      </c>
+      <c r="N66" s="111" t="n">
+        <v>46221</v>
       </c>
       <c r="O66" s="30" t="inlineStr">
         <is>
@@ -5760,11 +5820,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M67" s="38" t="n">
-        <v>46185</v>
-      </c>
-      <c r="N67" s="38" t="n">
-        <v>46195</v>
+      <c r="M67" s="111" t="n">
+        <v>46215</v>
+      </c>
+      <c r="N67" s="111" t="n">
+        <v>46225</v>
       </c>
       <c r="O67" s="30" t="inlineStr">
         <is>
@@ -5835,11 +5895,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M68" s="38" t="n">
-        <v>46185</v>
-      </c>
-      <c r="N68" s="38" t="n">
-        <v>46195</v>
+      <c r="M68" s="111" t="n">
+        <v>46215</v>
+      </c>
+      <c r="N68" s="111" t="n">
+        <v>46225</v>
       </c>
       <c r="O68" s="30" t="inlineStr">
         <is>
@@ -5910,11 +5970,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M69" s="38" t="n">
-        <v>46185</v>
-      </c>
-      <c r="N69" s="38" t="n">
-        <v>46195</v>
+      <c r="M69" s="111" t="n">
+        <v>46215</v>
+      </c>
+      <c r="N69" s="111" t="n">
+        <v>46225</v>
       </c>
       <c r="O69" s="30" t="inlineStr">
         <is>
@@ -5985,11 +6045,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M70" s="38" t="n">
-        <v>46187</v>
-      </c>
-      <c r="N70" s="38" t="n">
-        <v>46195</v>
+      <c r="M70" s="111" t="n">
+        <v>46217</v>
+      </c>
+      <c r="N70" s="111" t="n">
+        <v>46225</v>
       </c>
       <c r="O70" s="30" t="inlineStr">
         <is>
@@ -6060,11 +6120,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M71" s="38" t="n">
-        <v>46191</v>
-      </c>
-      <c r="N71" s="38" t="n">
-        <v>46198</v>
+      <c r="M71" s="111" t="n">
+        <v>46221</v>
+      </c>
+      <c r="N71" s="111" t="n">
+        <v>46228</v>
       </c>
       <c r="O71" s="30" t="inlineStr">
         <is>
@@ -6135,11 +6195,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M72" s="38" t="n">
-        <v>46193</v>
-      </c>
-      <c r="N72" s="38" t="n">
-        <v>46200</v>
+      <c r="M72" s="111" t="n">
+        <v>46223</v>
+      </c>
+      <c r="N72" s="111" t="n">
+        <v>46230</v>
       </c>
       <c r="O72" s="30" t="inlineStr">
         <is>
@@ -6210,11 +6270,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M73" s="38" t="n">
-        <v>46193</v>
-      </c>
-      <c r="N73" s="38" t="n">
-        <v>46203</v>
+      <c r="M73" s="111" t="n">
+        <v>46223</v>
+      </c>
+      <c r="N73" s="111" t="n">
+        <v>46233</v>
       </c>
       <c r="O73" s="30" t="inlineStr">
         <is>
@@ -6285,11 +6345,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M74" s="38" t="n">
-        <v>46195</v>
-      </c>
-      <c r="N74" s="38" t="n">
-        <v>46203</v>
+      <c r="M74" s="111" t="n">
+        <v>46225</v>
+      </c>
+      <c r="N74" s="111" t="n">
+        <v>46233</v>
       </c>
       <c r="O74" s="30" t="inlineStr">
         <is>
@@ -6360,11 +6420,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M75" s="38" t="n">
-        <v>46198</v>
-      </c>
-      <c r="N75" s="38" t="n">
-        <v>46205</v>
+      <c r="M75" s="111" t="n">
+        <v>46228</v>
+      </c>
+      <c r="N75" s="111" t="n">
+        <v>46235</v>
       </c>
       <c r="O75" s="30" t="inlineStr">
         <is>
@@ -6435,11 +6495,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M76" s="38" t="n">
-        <v>46198</v>
-      </c>
-      <c r="N76" s="38" t="n">
-        <v>46205</v>
+      <c r="M76" s="111" t="n">
+        <v>46228</v>
+      </c>
+      <c r="N76" s="111" t="n">
+        <v>46235</v>
       </c>
       <c r="O76" s="30" t="inlineStr">
         <is>
@@ -6510,11 +6570,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M77" s="38" t="n">
-        <v>46201</v>
-      </c>
-      <c r="N77" s="38" t="n">
-        <v>46208</v>
+      <c r="M77" s="111" t="n">
+        <v>46231</v>
+      </c>
+      <c r="N77" s="111" t="n">
+        <v>46238</v>
       </c>
       <c r="O77" s="30" t="inlineStr">
         <is>
@@ -6585,11 +6645,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M78" s="38" t="n">
-        <v>46205</v>
-      </c>
-      <c r="N78" s="38" t="n">
-        <v>46210</v>
+      <c r="M78" s="111" t="n">
+        <v>46235</v>
+      </c>
+      <c r="N78" s="111" t="n">
+        <v>46240</v>
       </c>
       <c r="O78" s="30" t="inlineStr">
         <is>
@@ -6660,11 +6720,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M79" s="38" t="n">
-        <v>46208</v>
-      </c>
-      <c r="N79" s="38" t="n">
-        <v>46215</v>
+      <c r="M79" s="111" t="n">
+        <v>46238</v>
+      </c>
+      <c r="N79" s="111" t="n">
+        <v>46245</v>
       </c>
       <c r="O79" s="30" t="inlineStr">
         <is>
@@ -6735,11 +6795,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M80" s="38" t="n">
-        <v>46210</v>
-      </c>
-      <c r="N80" s="38" t="n">
-        <v>46218</v>
+      <c r="M80" s="111" t="n">
+        <v>46240</v>
+      </c>
+      <c r="N80" s="111" t="n">
+        <v>46248</v>
       </c>
       <c r="O80" s="30" t="inlineStr">
         <is>
@@ -6810,11 +6870,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M81" s="38" t="n">
-        <v>46215</v>
-      </c>
-      <c r="N81" s="38" t="n">
-        <v>46234</v>
+      <c r="M81" s="111" t="n">
+        <v>46245</v>
+      </c>
+      <c r="N81" s="111" t="n">
+        <v>46264</v>
       </c>
       <c r="O81" s="30" t="inlineStr">
         <is>
@@ -6832,21 +6892,21 @@
           <t>PHASE 3 — IMPLEMENTATION (Hybrid)</t>
         </is>
       </c>
-      <c r="B82" s="3" t="n"/>
-      <c r="C82" s="3" t="n"/>
-      <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
-      <c r="F82" s="3" t="n"/>
-      <c r="G82" s="3" t="n"/>
-      <c r="H82" s="3" t="n"/>
-      <c r="I82" s="3" t="n"/>
-      <c r="J82" s="3" t="n"/>
-      <c r="K82" s="3" t="n"/>
-      <c r="L82" s="3" t="n"/>
-      <c r="M82" s="3" t="n"/>
-      <c r="N82" s="3" t="n"/>
-      <c r="O82" s="3" t="n"/>
-      <c r="P82" s="3" t="n"/>
+      <c r="B82" s="107" t="n"/>
+      <c r="C82" s="107" t="n"/>
+      <c r="D82" s="107" t="n"/>
+      <c r="E82" s="107" t="n"/>
+      <c r="F82" s="107" t="n"/>
+      <c r="G82" s="107" t="n"/>
+      <c r="H82" s="107" t="n"/>
+      <c r="I82" s="107" t="n"/>
+      <c r="J82" s="107" t="n"/>
+      <c r="K82" s="107" t="n"/>
+      <c r="L82" s="107" t="n"/>
+      <c r="M82" s="107" t="n"/>
+      <c r="N82" s="107" t="n"/>
+      <c r="O82" s="107" t="n"/>
+      <c r="P82" s="108" t="n"/>
     </row>
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="43" t="n">
@@ -6907,11 +6967,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M83" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="N83" s="52" t="n">
-        <v>46233</v>
+      <c r="M83" s="112" t="n">
+        <v>46266</v>
+      </c>
+      <c r="N83" s="112" t="n">
+        <v>46281</v>
       </c>
       <c r="O83" s="43" t="inlineStr">
         <is>
@@ -6982,11 +7042,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M84" s="52" t="n">
-        <v>46223</v>
-      </c>
-      <c r="N84" s="52" t="n">
-        <v>46239</v>
+      <c r="M84" s="112" t="n">
+        <v>46271</v>
+      </c>
+      <c r="N84" s="112" t="n">
+        <v>46286</v>
       </c>
       <c r="O84" s="43" t="inlineStr">
         <is>
@@ -7057,11 +7117,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M85" s="52" t="n">
-        <v>46228</v>
-      </c>
-      <c r="N85" s="52" t="n">
-        <v>46244</v>
+      <c r="M85" s="112" t="n">
+        <v>46276</v>
+      </c>
+      <c r="N85" s="112" t="n">
+        <v>46291</v>
       </c>
       <c r="O85" s="43" t="inlineStr">
         <is>
@@ -7132,11 +7192,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M86" s="52" t="n">
-        <v>46218</v>
-      </c>
-      <c r="N86" s="52" t="n">
-        <v>46239</v>
+      <c r="M86" s="112" t="n">
+        <v>46266</v>
+      </c>
+      <c r="N86" s="112" t="n">
+        <v>46286</v>
       </c>
       <c r="O86" s="43" t="inlineStr">
         <is>
@@ -7207,11 +7267,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M87" s="52" t="n">
-        <v>46235</v>
-      </c>
-      <c r="N87" s="52" t="n">
-        <v>46249</v>
+      <c r="M87" s="112" t="n">
+        <v>46283</v>
+      </c>
+      <c r="N87" s="112" t="n">
+        <v>46296</v>
       </c>
       <c r="O87" s="43" t="inlineStr">
         <is>
@@ -7282,11 +7342,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M88" s="52" t="n">
-        <v>46239</v>
-      </c>
-      <c r="N88" s="52" t="n">
-        <v>46259</v>
+      <c r="M88" s="112" t="n">
+        <v>46286</v>
+      </c>
+      <c r="N88" s="112" t="n">
+        <v>46306</v>
       </c>
       <c r="O88" s="43" t="inlineStr">
         <is>
@@ -7357,11 +7417,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M89" s="52" t="n">
-        <v>46235</v>
-      </c>
-      <c r="N89" s="52" t="n">
-        <v>46264</v>
+      <c r="M89" s="112" t="n">
+        <v>46283</v>
+      </c>
+      <c r="N89" s="112" t="n">
+        <v>46311</v>
       </c>
       <c r="O89" s="43" t="inlineStr">
         <is>
@@ -7432,11 +7492,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M90" s="52" t="n">
-        <v>46223</v>
-      </c>
-      <c r="N90" s="52" t="n">
-        <v>46249</v>
+      <c r="M90" s="112" t="n">
+        <v>46271</v>
+      </c>
+      <c r="N90" s="112" t="n">
+        <v>46296</v>
       </c>
       <c r="O90" s="43" t="inlineStr">
         <is>
@@ -7507,11 +7567,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M91" s="52" t="n">
-        <v>46244</v>
-      </c>
-      <c r="N91" s="52" t="n">
-        <v>46270</v>
+      <c r="M91" s="112" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N91" s="112" t="n">
+        <v>46317</v>
       </c>
       <c r="O91" s="43" t="inlineStr">
         <is>
@@ -7582,11 +7642,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M92" s="52" t="n">
-        <v>46235</v>
-      </c>
-      <c r="N92" s="52" t="n">
-        <v>46254</v>
+      <c r="M92" s="112" t="n">
+        <v>46283</v>
+      </c>
+      <c r="N92" s="112" t="n">
+        <v>46301</v>
       </c>
       <c r="O92" s="43" t="inlineStr">
         <is>
@@ -7657,11 +7717,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M93" s="52" t="n">
-        <v>46249</v>
-      </c>
-      <c r="N93" s="52" t="n">
-        <v>46280</v>
+      <c r="M93" s="112" t="n">
+        <v>46296</v>
+      </c>
+      <c r="N93" s="112" t="n">
+        <v>46326</v>
       </c>
       <c r="O93" s="43" t="inlineStr">
         <is>
@@ -7732,11 +7792,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M94" s="52" t="n">
-        <v>46254</v>
-      </c>
-      <c r="N94" s="52" t="n">
-        <v>46275</v>
+      <c r="M94" s="112" t="n">
+        <v>46301</v>
+      </c>
+      <c r="N94" s="112" t="n">
+        <v>46321</v>
       </c>
       <c r="O94" s="43" t="inlineStr">
         <is>
@@ -7807,11 +7867,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M95" s="52" t="n">
-        <v>46249</v>
-      </c>
-      <c r="N95" s="52" t="n">
-        <v>46295</v>
+      <c r="M95" s="112" t="n">
+        <v>46296</v>
+      </c>
+      <c r="N95" s="112" t="n">
+        <v>46341</v>
       </c>
       <c r="O95" s="43" t="inlineStr">
         <is>
@@ -7882,11 +7942,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M96" s="52" t="n">
-        <v>46259</v>
-      </c>
-      <c r="N96" s="52" t="n">
-        <v>46310</v>
+      <c r="M96" s="112" t="n">
+        <v>46306</v>
+      </c>
+      <c r="N96" s="112" t="n">
+        <v>46355</v>
       </c>
       <c r="O96" s="43" t="inlineStr">
         <is>
@@ -7957,11 +8017,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M97" s="52" t="n">
-        <v>46235</v>
-      </c>
-      <c r="N97" s="52" t="n">
-        <v>46254</v>
+      <c r="M97" s="112" t="n">
+        <v>46283</v>
+      </c>
+      <c r="N97" s="112" t="n">
+        <v>46301</v>
       </c>
       <c r="O97" s="43" t="inlineStr">
         <is>
@@ -8032,11 +8092,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M98" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N98" s="52" t="n">
-        <v>46310</v>
+      <c r="M98" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N98" s="112" t="n">
+        <v>46355</v>
       </c>
       <c r="O98" s="43" t="inlineStr">
         <is>
@@ -8107,11 +8167,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M99" s="52" t="n">
-        <v>46249</v>
-      </c>
-      <c r="N99" s="52" t="n">
-        <v>46270</v>
+      <c r="M99" s="112" t="n">
+        <v>46296</v>
+      </c>
+      <c r="N99" s="112" t="n">
+        <v>46317</v>
       </c>
       <c r="O99" s="43" t="inlineStr">
         <is>
@@ -8182,11 +8242,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M100" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N100" s="52" t="n">
-        <v>46295</v>
+      <c r="M100" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N100" s="112" t="n">
+        <v>46341</v>
       </c>
       <c r="O100" s="43" t="inlineStr">
         <is>
@@ -8257,11 +8317,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M101" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N101" s="52" t="n">
-        <v>46285</v>
+      <c r="M101" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N101" s="112" t="n">
+        <v>46331</v>
       </c>
       <c r="O101" s="43" t="inlineStr">
         <is>
@@ -8332,11 +8392,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M102" s="52" t="n">
-        <v>46270</v>
-      </c>
-      <c r="N102" s="52" t="n">
-        <v>46290</v>
+      <c r="M102" s="112" t="n">
+        <v>46317</v>
+      </c>
+      <c r="N102" s="112" t="n">
+        <v>46336</v>
       </c>
       <c r="O102" s="43" t="inlineStr">
         <is>
@@ -8407,11 +8467,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M103" s="52" t="n">
-        <v>46285</v>
-      </c>
-      <c r="N103" s="52" t="n">
-        <v>46310</v>
+      <c r="M103" s="112" t="n">
+        <v>46331</v>
+      </c>
+      <c r="N103" s="112" t="n">
+        <v>46355</v>
       </c>
       <c r="O103" s="43" t="inlineStr">
         <is>
@@ -8482,11 +8542,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M104" s="52" t="n">
-        <v>46223</v>
-      </c>
-      <c r="N104" s="52" t="n">
-        <v>46244</v>
+      <c r="M104" s="112" t="n">
+        <v>46271</v>
+      </c>
+      <c r="N104" s="112" t="n">
+        <v>46291</v>
       </c>
       <c r="O104" s="43" t="inlineStr">
         <is>
@@ -8557,11 +8617,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M105" s="52" t="n">
-        <v>46244</v>
-      </c>
-      <c r="N105" s="52" t="n">
-        <v>46264</v>
+      <c r="M105" s="112" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N105" s="112" t="n">
+        <v>46311</v>
       </c>
       <c r="O105" s="43" t="inlineStr">
         <is>
@@ -8632,11 +8692,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M106" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N106" s="52" t="n">
-        <v>46310</v>
+      <c r="M106" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N106" s="112" t="n">
+        <v>46355</v>
       </c>
       <c r="O106" s="43" t="inlineStr">
         <is>
@@ -8707,11 +8767,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M107" s="52" t="n">
-        <v>46235</v>
-      </c>
-      <c r="N107" s="52" t="n">
-        <v>46254</v>
+      <c r="M107" s="112" t="n">
+        <v>46283</v>
+      </c>
+      <c r="N107" s="112" t="n">
+        <v>46301</v>
       </c>
       <c r="O107" s="43" t="inlineStr">
         <is>
@@ -8782,11 +8842,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M108" s="52" t="n">
-        <v>46254</v>
-      </c>
-      <c r="N108" s="52" t="n">
-        <v>46275</v>
+      <c r="M108" s="112" t="n">
+        <v>46301</v>
+      </c>
+      <c r="N108" s="112" t="n">
+        <v>46321</v>
       </c>
       <c r="O108" s="43" t="inlineStr">
         <is>
@@ -8857,11 +8917,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M109" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N109" s="52" t="n">
-        <v>46295</v>
+      <c r="M109" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N109" s="112" t="n">
+        <v>46341</v>
       </c>
       <c r="O109" s="43" t="inlineStr">
         <is>
@@ -8932,11 +8992,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M110" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N110" s="52" t="n">
-        <v>46295</v>
+      <c r="M110" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N110" s="112" t="n">
+        <v>46341</v>
       </c>
       <c r="O110" s="43" t="inlineStr">
         <is>
@@ -9007,11 +9067,11 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M111" s="52" t="n">
-        <v>46223</v>
-      </c>
-      <c r="N111" s="52" t="n">
-        <v>46239</v>
+      <c r="M111" s="112" t="n">
+        <v>46271</v>
+      </c>
+      <c r="N111" s="112" t="n">
+        <v>46286</v>
       </c>
       <c r="O111" s="43" t="inlineStr">
         <is>
@@ -9082,11 +9142,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M112" s="52" t="n">
-        <v>46249</v>
-      </c>
-      <c r="N112" s="52" t="n">
-        <v>46326</v>
+      <c r="M112" s="112" t="n">
+        <v>46296</v>
+      </c>
+      <c r="N112" s="112" t="n">
+        <v>46371</v>
       </c>
       <c r="O112" s="43" t="inlineStr">
         <is>
@@ -9157,11 +9217,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M113" s="52" t="n">
-        <v>46235</v>
-      </c>
-      <c r="N113" s="52" t="n">
-        <v>46259</v>
+      <c r="M113" s="112" t="n">
+        <v>46283</v>
+      </c>
+      <c r="N113" s="112" t="n">
+        <v>46306</v>
       </c>
       <c r="O113" s="43" t="inlineStr">
         <is>
@@ -9232,11 +9292,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M114" s="52" t="n">
-        <v>46259</v>
-      </c>
-      <c r="N114" s="52" t="n">
-        <v>46270</v>
+      <c r="M114" s="112" t="n">
+        <v>46306</v>
+      </c>
+      <c r="N114" s="112" t="n">
+        <v>46317</v>
       </c>
       <c r="O114" s="43" t="inlineStr">
         <is>
@@ -9307,11 +9367,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M115" s="52" t="n">
-        <v>46244</v>
-      </c>
-      <c r="N115" s="52" t="n">
-        <v>46266</v>
+      <c r="M115" s="112" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N115" s="112" t="n">
+        <v>46313</v>
       </c>
       <c r="O115" s="43" t="inlineStr">
         <is>
@@ -9382,11 +9442,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M116" s="52" t="n">
-        <v>46249</v>
-      </c>
-      <c r="N116" s="52" t="n">
-        <v>46275</v>
+      <c r="M116" s="112" t="n">
+        <v>46296</v>
+      </c>
+      <c r="N116" s="112" t="n">
+        <v>46321</v>
       </c>
       <c r="O116" s="43" t="inlineStr">
         <is>
@@ -9457,11 +9517,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M117" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N117" s="52" t="n">
-        <v>46285</v>
+      <c r="M117" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N117" s="112" t="n">
+        <v>46331</v>
       </c>
       <c r="O117" s="43" t="inlineStr">
         <is>
@@ -9532,11 +9592,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M118" s="52" t="n">
-        <v>46270</v>
-      </c>
-      <c r="N118" s="52" t="n">
-        <v>46290</v>
+      <c r="M118" s="112" t="n">
+        <v>46317</v>
+      </c>
+      <c r="N118" s="112" t="n">
+        <v>46336</v>
       </c>
       <c r="O118" s="43" t="inlineStr">
         <is>
@@ -9607,11 +9667,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M119" s="52" t="n">
-        <v>46249</v>
-      </c>
-      <c r="N119" s="52" t="n">
-        <v>46295</v>
+      <c r="M119" s="112" t="n">
+        <v>46296</v>
+      </c>
+      <c r="N119" s="112" t="n">
+        <v>46341</v>
       </c>
       <c r="O119" s="43" t="inlineStr">
         <is>
@@ -9682,11 +9742,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M120" s="52" t="n">
-        <v>46266</v>
-      </c>
-      <c r="N120" s="52" t="n">
-        <v>46310</v>
+      <c r="M120" s="112" t="n">
+        <v>46313</v>
+      </c>
+      <c r="N120" s="112" t="n">
+        <v>46355</v>
       </c>
       <c r="O120" s="43" t="inlineStr">
         <is>
@@ -9757,11 +9817,11 @@
           <t>CREATE</t>
         </is>
       </c>
-      <c r="M121" s="52" t="n">
-        <v>46280</v>
-      </c>
-      <c r="N121" s="52" t="n">
-        <v>46325</v>
+      <c r="M121" s="112" t="n">
+        <v>46326</v>
+      </c>
+      <c r="N121" s="112" t="n">
+        <v>46370</v>
       </c>
       <c r="O121" s="43" t="inlineStr">
         <is>
@@ -9779,21 +9839,21 @@
           <t>PHASE 4 — STABILIZATION &amp; ADVISORY (Remote)</t>
         </is>
       </c>
-      <c r="B122" s="3" t="n"/>
-      <c r="C122" s="3" t="n"/>
-      <c r="D122" s="3" t="n"/>
-      <c r="E122" s="3" t="n"/>
-      <c r="F122" s="3" t="n"/>
-      <c r="G122" s="3" t="n"/>
-      <c r="H122" s="3" t="n"/>
-      <c r="I122" s="3" t="n"/>
-      <c r="J122" s="3" t="n"/>
-      <c r="K122" s="3" t="n"/>
-      <c r="L122" s="3" t="n"/>
-      <c r="M122" s="3" t="n"/>
-      <c r="N122" s="3" t="n"/>
-      <c r="O122" s="3" t="n"/>
-      <c r="P122" s="3" t="n"/>
+      <c r="B122" s="107" t="n"/>
+      <c r="C122" s="107" t="n"/>
+      <c r="D122" s="107" t="n"/>
+      <c r="E122" s="107" t="n"/>
+      <c r="F122" s="107" t="n"/>
+      <c r="G122" s="107" t="n"/>
+      <c r="H122" s="107" t="n"/>
+      <c r="I122" s="107" t="n"/>
+      <c r="J122" s="107" t="n"/>
+      <c r="K122" s="107" t="n"/>
+      <c r="L122" s="107" t="n"/>
+      <c r="M122" s="107" t="n"/>
+      <c r="N122" s="107" t="n"/>
+      <c r="O122" s="107" t="n"/>
+      <c r="P122" s="108" t="n"/>
     </row>
     <row r="123" ht="28" customHeight="1">
       <c r="A123" s="56" t="n">
@@ -9854,11 +9914,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M123" s="64" t="n">
-        <v>46327</v>
-      </c>
-      <c r="N123" s="64" t="n">
-        <v>46341</v>
+      <c r="M123" s="113" t="n">
+        <v>46388</v>
+      </c>
+      <c r="N123" s="113" t="n">
+        <v>46398</v>
       </c>
       <c r="O123" s="56" t="inlineStr">
         <is>
@@ -9929,11 +9989,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M124" s="64" t="n">
-        <v>46336</v>
-      </c>
-      <c r="N124" s="64" t="n">
-        <v>46346</v>
+      <c r="M124" s="113" t="n">
+        <v>46395</v>
+      </c>
+      <c r="N124" s="113" t="n">
+        <v>46402</v>
       </c>
       <c r="O124" s="56" t="inlineStr">
         <is>
@@ -10004,11 +10064,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M125" s="64" t="n">
-        <v>46341</v>
-      </c>
-      <c r="N125" s="64" t="n">
-        <v>46356</v>
+      <c r="M125" s="113" t="n">
+        <v>46398</v>
+      </c>
+      <c r="N125" s="113" t="n">
+        <v>46410</v>
       </c>
       <c r="O125" s="56" t="inlineStr">
         <is>
@@ -10079,11 +10139,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M126" s="64" t="n">
-        <v>46346</v>
-      </c>
-      <c r="N126" s="64" t="n">
-        <v>46371</v>
+      <c r="M126" s="113" t="n">
+        <v>46402</v>
+      </c>
+      <c r="N126" s="113" t="n">
+        <v>46421</v>
       </c>
       <c r="O126" s="56" t="inlineStr">
         <is>
@@ -10154,11 +10214,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M127" s="64" t="n">
-        <v>46341</v>
-      </c>
-      <c r="N127" s="64" t="n">
-        <v>46371</v>
+      <c r="M127" s="113" t="n">
+        <v>46398</v>
+      </c>
+      <c r="N127" s="113" t="n">
+        <v>46421</v>
       </c>
       <c r="O127" s="56" t="inlineStr">
         <is>
@@ -10229,11 +10289,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M128" s="64" t="n">
-        <v>46327</v>
-      </c>
-      <c r="N128" s="64" t="n">
-        <v>46356</v>
+      <c r="M128" s="113" t="n">
+        <v>46388</v>
+      </c>
+      <c r="N128" s="113" t="n">
+        <v>46410</v>
       </c>
       <c r="O128" s="56" t="inlineStr">
         <is>
@@ -10304,11 +10364,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M129" s="64" t="n">
-        <v>46336</v>
-      </c>
-      <c r="N129" s="64" t="n">
-        <v>46356</v>
+      <c r="M129" s="113" t="n">
+        <v>46395</v>
+      </c>
+      <c r="N129" s="113" t="n">
+        <v>46410</v>
       </c>
       <c r="O129" s="56" t="inlineStr">
         <is>
@@ -10379,11 +10439,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M130" s="64" t="n">
-        <v>46341</v>
-      </c>
-      <c r="N130" s="64" t="n">
-        <v>46361</v>
+      <c r="M130" s="113" t="n">
+        <v>46398</v>
+      </c>
+      <c r="N130" s="113" t="n">
+        <v>46413</v>
       </c>
       <c r="O130" s="56" t="inlineStr">
         <is>
@@ -10454,11 +10514,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M131" s="64" t="n">
-        <v>46351</v>
-      </c>
-      <c r="N131" s="64" t="n">
-        <v>46366</v>
+      <c r="M131" s="113" t="n">
+        <v>46406</v>
+      </c>
+      <c r="N131" s="113" t="n">
+        <v>46417</v>
       </c>
       <c r="O131" s="56" t="inlineStr">
         <is>
@@ -10529,11 +10589,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M132" s="64" t="n">
-        <v>46366</v>
-      </c>
-      <c r="N132" s="64" t="n">
-        <v>46371</v>
+      <c r="M132" s="113" t="n">
+        <v>46417</v>
+      </c>
+      <c r="N132" s="113" t="n">
+        <v>46421</v>
       </c>
       <c r="O132" s="56" t="inlineStr">
         <is>
@@ -10604,11 +10664,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M133" s="64" t="n">
-        <v>46341</v>
-      </c>
-      <c r="N133" s="64" t="n">
-        <v>46371</v>
+      <c r="M133" s="113" t="n">
+        <v>46398</v>
+      </c>
+      <c r="N133" s="113" t="n">
+        <v>46421</v>
       </c>
       <c r="O133" s="56" t="inlineStr">
         <is>
@@ -10679,11 +10739,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M134" s="64" t="n">
-        <v>46346</v>
-      </c>
-      <c r="N134" s="64" t="n">
-        <v>46376</v>
+      <c r="M134" s="113" t="n">
+        <v>46402</v>
+      </c>
+      <c r="N134" s="113" t="n">
+        <v>46425</v>
       </c>
       <c r="O134" s="56" t="inlineStr">
         <is>
@@ -10754,11 +10814,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M135" s="64" t="n">
-        <v>46341</v>
-      </c>
-      <c r="N135" s="64" t="n">
-        <v>46366</v>
+      <c r="M135" s="113" t="n">
+        <v>46398</v>
+      </c>
+      <c r="N135" s="113" t="n">
+        <v>46417</v>
       </c>
       <c r="O135" s="56" t="inlineStr">
         <is>
@@ -10829,11 +10889,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M136" s="64" t="n">
-        <v>46357</v>
-      </c>
-      <c r="N136" s="64" t="n">
-        <v>46376</v>
+      <c r="M136" s="113" t="n">
+        <v>46410</v>
+      </c>
+      <c r="N136" s="113" t="n">
+        <v>46425</v>
       </c>
       <c r="O136" s="56" t="inlineStr">
         <is>
@@ -10904,11 +10964,11 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M137" s="64" t="n">
-        <v>46341</v>
-      </c>
-      <c r="N137" s="64" t="n">
-        <v>46371</v>
+      <c r="M137" s="113" t="n">
+        <v>46398</v>
+      </c>
+      <c r="N137" s="113" t="n">
+        <v>46421</v>
       </c>
       <c r="O137" s="56" t="inlineStr">
         <is>
@@ -10979,11 +11039,11 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M138" s="64" t="n">
-        <v>46357</v>
-      </c>
-      <c r="N138" s="64" t="n">
-        <v>46376</v>
+      <c r="M138" s="113" t="n">
+        <v>46410</v>
+      </c>
+      <c r="N138" s="113" t="n">
+        <v>46425</v>
       </c>
       <c r="O138" s="56" t="inlineStr">
         <is>
@@ -11054,11 +11114,11 @@
           <t>BUILD</t>
         </is>
       </c>
-      <c r="M139" s="64" t="n">
-        <v>46361</v>
-      </c>
-      <c r="N139" s="64" t="n">
-        <v>46376</v>
+      <c r="M139" s="113" t="n">
+        <v>46413</v>
+      </c>
+      <c r="N139" s="113" t="n">
+        <v>46425</v>
       </c>
       <c r="O139" s="56" t="inlineStr">
         <is>
@@ -11129,11 +11189,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M140" s="64" t="n">
-        <v>46361</v>
-      </c>
-      <c r="N140" s="64" t="n">
-        <v>46376</v>
+      <c r="M140" s="113" t="n">
+        <v>46413</v>
+      </c>
+      <c r="N140" s="113" t="n">
+        <v>46425</v>
       </c>
       <c r="O140" s="56" t="inlineStr">
         <is>
@@ -11204,11 +11264,11 @@
           <t>EXECUTE</t>
         </is>
       </c>
-      <c r="M141" s="64" t="n">
-        <v>46366</v>
-      </c>
-      <c r="N141" s="64" t="n">
-        <v>46376</v>
+      <c r="M141" s="113" t="n">
+        <v>46417</v>
+      </c>
+      <c r="N141" s="113" t="n">
+        <v>46425</v>
       </c>
       <c r="O141" s="56" t="inlineStr">
         <is>
@@ -11279,10 +11339,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M142" s="64" t="n">
-        <v>46388</v>
-      </c>
-      <c r="N142" s="64" t="n">
+      <c r="M142" s="113" t="n">
+        <v>46434</v>
+      </c>
+      <c r="N142" s="113" t="n">
         <v>46568</v>
       </c>
       <c r="O142" s="56" t="inlineStr">
@@ -11354,10 +11414,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M143" s="64" t="n">
-        <v>46388</v>
-      </c>
-      <c r="N143" s="64" t="n">
+      <c r="M143" s="113" t="n">
+        <v>46434</v>
+      </c>
+      <c r="N143" s="113" t="n">
         <v>46568</v>
       </c>
       <c r="O143" s="56" t="inlineStr">
@@ -11429,10 +11489,10 @@
           <t>ALL</t>
         </is>
       </c>
-      <c r="M144" s="64" t="n">
-        <v>46539</v>
-      </c>
-      <c r="N144" s="64" t="n">
+      <c r="M144" s="113" t="n">
+        <v>46546</v>
+      </c>
+      <c r="N144" s="113" t="n">
         <v>46568</v>
       </c>
       <c r="O144" s="56" t="inlineStr">
@@ -11481,6 +11541,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -11549,7 +11610,7 @@
       </c>
       <c r="B5" s="75" t="inlineStr">
         <is>
-          <t>May 1 – May 30, 2026</t>
+          <t>May 1 – Jun 30, 2026</t>
         </is>
       </c>
       <c r="C5" s="75" t="inlineStr">
@@ -11577,7 +11638,7 @@
       </c>
       <c r="B6" s="80" t="inlineStr">
         <is>
-          <t>Jun 1 – Jul 31, 2026</t>
+          <t>Jul 1 – Aug 31, 2026</t>
         </is>
       </c>
       <c r="C6" s="80" t="inlineStr">
@@ -11605,7 +11666,7 @@
       </c>
       <c r="B7" s="85" t="inlineStr">
         <is>
-          <t>Jul 15 – Oct 31, 2026</t>
+          <t>Sep 1 – Dec 15, 2026</t>
         </is>
       </c>
       <c r="C7" s="85" t="inlineStr">
@@ -11633,7 +11694,7 @@
       </c>
       <c r="B8" s="90" t="inlineStr">
         <is>
-          <t>Nov 1, 2026 – Jun 30, 2027</t>
+          <t>Jan 1 – Jun 30, 2027</t>
         </is>
       </c>
       <c r="C8" s="90" t="inlineStr">
@@ -11669,6 +11730,7 @@
       </c>
       <c r="F9" s="95" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="98" t="inlineStr">
         <is>
@@ -11768,6 +11830,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="98" t="inlineStr">
         <is>

</xml_diff>